<commit_message>
feat: implement core configuration types and schema loading infrastructure for protocol definitions
</commit_message>
<xml_diff>
--- a/DB_48100.xlsx
+++ b/DB_48100.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\Python\Bytehound\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA3DD00-D2A8-4BE9-965F-D0E0A46EF1DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BACBC8B-C9AE-480B-A05A-F59D10500F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="182">
   <si>
     <t>id_or_address</t>
   </si>
@@ -568,9 +568,6 @@
     <t>CC_SOC</t>
   </si>
   <si>
-    <t>``````</t>
-  </si>
-  <si>
     <t>SOC</t>
   </si>
   <si>
@@ -581,6 +578,15 @@
   </si>
   <si>
     <t>Capacity</t>
+  </si>
+  <si>
+    <t>0x1F3</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>Error</t>
   </si>
 </sst>
 </file>
@@ -1047,7 +1053,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="36.1796875" bestFit="1" customWidth="1"/>
@@ -1296,6 +1302,23 @@
         <v>1</v>
       </c>
     </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>179</v>
+      </c>
+      <c r="B15" t="s">
+        <v>180</v>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+      <c r="D15" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1303,7 +1326,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
@@ -2066,7 +2089,7 @@
         <v>173</v>
       </c>
       <c r="I18" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J18" t="s">
         <v>23</v>
@@ -2104,7 +2127,7 @@
         <v>173</v>
       </c>
       <c r="I19" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J19" t="s">
         <v>23</v>
@@ -2121,7 +2144,7 @@
         <v>169</v>
       </c>
       <c r="B20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C20" t="s">
         <v>172</v>
@@ -2139,10 +2162,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="s">
+        <v>177</v>
+      </c>
+      <c r="I20" t="s">
         <v>178</v>
-      </c>
-      <c r="I20" t="s">
-        <v>179</v>
       </c>
       <c r="J20" t="s">
         <v>23</v>
@@ -2154,9 +2177,42 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="L23" t="s">
-        <v>175</v>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>179</v>
+      </c>
+      <c r="B21" t="s">
+        <v>181</v>
+      </c>
+      <c r="C21" t="s">
+        <v>172</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21" t="s">
+        <v>177</v>
+      </c>
+      <c r="I21" t="s">
+        <v>178</v>
+      </c>
+      <c r="J21" t="s">
+        <v>23</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="N21" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>